<commit_message>
updates from first survey results round
</commit_message>
<xml_diff>
--- a/Standards/Templates/Template.xlsx
+++ b/Standards/Templates/Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mahnoorzulfiqar/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/zimmermann/Members/zulfiqar/ZM009_NFDI4Micro/003_Experiments/DataAnalysis/ZM009A_DryLab/Standards/Templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{744B55CF-ADE3-F247-8455-14AEF7772602}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7246659-9361-5A47-8D2A-2C3D7FE8F700}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2540" yWindow="840" windowWidth="13880" windowHeight="19920" activeTab="5" xr2:uid="{7929348A-0049-9D47-B318-DD8A1A5D02A5}"/>
+    <workbookView xWindow="34060" yWindow="4260" windowWidth="32020" windowHeight="19840" activeTab="2" xr2:uid="{7929348A-0049-9D47-B318-DD8A1A5D02A5}"/>
   </bookViews>
   <sheets>
     <sheet name="Template_Description" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="294">
   <si>
     <t>SMILES</t>
   </si>
@@ -343,9 +343,6 @@
     <t>Sample preparation</t>
   </si>
   <si>
-    <t>Kinetic parameters</t>
-  </si>
-  <si>
     <t xml:space="preserve">Activity type </t>
   </si>
   <si>
@@ -373,12 +370,6 @@
     <t>ACTIVITY_COMMENT</t>
   </si>
   <si>
-    <t>If you would like to only report a text rather than a numerical valaue, make sure to stick to your own defined vocabulary here. We recommend to fill the VALUE and its related fields as best practice</t>
-  </si>
-  <si>
-    <t>The numerical value of the activity measurement (see TEXT_VALUE for non-numerical values); please keep TEXT_VALUE empty if you plan to fill this column</t>
-  </si>
-  <si>
     <t>UPPER_VALUE</t>
   </si>
   <si>
@@ -905,6 +896,42 @@
   </si>
   <si>
     <t>hydorlysis</t>
+  </si>
+  <si>
+    <t>The numerical value of the activity measurement (see TEXT_VALUE for non-numerical values); please keep TEXT_VALUE empty if you plan to fill this column. E.g: here you can add IC50, EC50, % biotransformation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">If you would like to only report a text rather than a numerical valaue, make sure to stick to your own defined vocabulary here. We recommend to fill the VALUE and its related fields as best practice. The lack of activity should be evident from this section. </t>
+  </si>
+  <si>
+    <t>Classify_activity</t>
+  </si>
+  <si>
+    <t>free value. Either you can label the activity as 0 - no activity and 1 - activity. Or you can write a comment with your defined thresholds</t>
+  </si>
+  <si>
+    <t>Kinetic_parameter_type</t>
+  </si>
+  <si>
+    <t>Kinetic_parameter_value</t>
+  </si>
+  <si>
+    <t>quantitative measures—that describe the rate, efficiency, and affinity of enzyme-catalyzed reactions. If available, write what type i.e. Km, Vmax, kcat</t>
+  </si>
+  <si>
+    <t>mention the value associated with the kinetic parameter mentioned before</t>
+  </si>
+  <si>
+    <t>Physicochemical properties columns</t>
+  </si>
+  <si>
+    <t>this could include logP, functional groups and the list goes. BioXend will automatically extract if not provided, choose: basic, extended, functional groups or all from the drop down menu</t>
+  </si>
+  <si>
+    <t>mzML file source</t>
+  </si>
+  <si>
+    <t>for MS2 fragmentation or as a source file to reproduce the rsults</t>
   </si>
 </sst>
 </file>
@@ -1165,7 +1192,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1217,7 +1244,6 @@
     <xf numFmtId="0" fontId="13" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="4" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1563,7 +1589,7 @@
     </row>
     <row r="2" spans="1:4" s="10" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="B2" s="11" t="s">
         <v>11</v>
@@ -1574,7 +1600,7 @@
     </row>
     <row r="3" spans="1:4" s="10" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="B3" s="11" t="s">
         <v>85</v>
@@ -1585,7 +1611,7 @@
     </row>
     <row r="4" spans="1:4" s="10" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="B4" s="11" t="s">
         <v>12</v>
@@ -1596,7 +1622,7 @@
     </row>
     <row r="5" spans="1:4" s="10" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B5" s="11" t="s">
         <v>13</v>
@@ -1607,7 +1633,7 @@
     </row>
     <row r="6" spans="1:4" s="8" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="B6" s="12" t="s">
         <v>14</v>
@@ -1618,7 +1644,7 @@
     </row>
     <row r="11" spans="1:4" ht="47" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
@@ -1626,26 +1652,26 @@
     </row>
     <row r="12" spans="1:4" ht="26" x14ac:dyDescent="0.3">
       <c r="B12" s="1" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="26" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="26" x14ac:dyDescent="0.3">
       <c r="B14" s="1" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="47" x14ac:dyDescent="0.55000000000000004">
@@ -1884,7 +1910,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13A45AA6-1501-444D-8DA9-A74997D7FE12}">
-  <dimension ref="A1:W4"/>
+  <dimension ref="A1:Y3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="25.83203125" style="25" customWidth="1"/>
@@ -1908,12 +1934,13 @@
     <col min="21" max="21" width="22.5" style="25" customWidth="1"/>
     <col min="22" max="22" width="33.33203125" style="25" customWidth="1"/>
     <col min="23" max="23" width="21.1640625" style="25" customWidth="1"/>
-    <col min="24" max="16384" width="10.83203125" style="25"/>
+    <col min="24" max="24" width="19.6640625" style="25" customWidth="1"/>
+    <col min="25" max="16384" width="10.83203125" style="25"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" s="17" customFormat="1" ht="88" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25" s="17" customFormat="1" ht="66" x14ac:dyDescent="0.25">
       <c r="A1" s="21" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B1" s="18" t="s">
         <v>1</v>
@@ -1925,19 +1952,19 @@
         <v>66</v>
       </c>
       <c r="E1" s="19" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="F1" s="19" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="G1" s="19" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H1" s="21" t="s">
         <v>65</v>
       </c>
       <c r="I1" s="19" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="J1" s="21" t="s">
         <v>2</v>
@@ -1949,128 +1976,140 @@
         <v>4</v>
       </c>
       <c r="M1" s="19" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="N1" s="19" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="O1" s="19" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="P1" s="19" t="s">
+        <v>141</v>
+      </c>
+      <c r="Q1" s="19" t="s">
+        <v>142</v>
+      </c>
+      <c r="R1" s="21" t="s">
         <v>144</v>
-      </c>
-      <c r="Q1" s="19" t="s">
-        <v>145</v>
-      </c>
-      <c r="R1" s="21" t="s">
-        <v>147</v>
       </c>
       <c r="S1" s="21" t="s">
         <v>5</v>
       </c>
       <c r="T1" s="21" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="U1" s="21" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="V1" s="21" t="s">
+        <v>202</v>
+      </c>
+      <c r="W1" s="21" t="s">
+        <v>204</v>
+      </c>
+      <c r="X1" s="19" t="s">
+        <v>290</v>
+      </c>
+      <c r="Y1" s="21" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="2" spans="1:25" s="26" customFormat="1" ht="220" x14ac:dyDescent="0.25">
+      <c r="A2" s="26" t="s">
+        <v>124</v>
+      </c>
+      <c r="B2" s="26" t="s">
+        <v>125</v>
+      </c>
+      <c r="C2" s="26" t="s">
+        <v>126</v>
+      </c>
+      <c r="D2" s="26" t="s">
+        <v>127</v>
+      </c>
+      <c r="E2" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="F2" s="26" t="s">
+        <v>138</v>
+      </c>
+      <c r="G2" s="26" t="s">
+        <v>139</v>
+      </c>
+      <c r="H2" s="26" t="s">
+        <v>129</v>
+      </c>
+      <c r="I2" s="26" t="s">
+        <v>130</v>
+      </c>
+      <c r="J2" s="26" t="s">
+        <v>131</v>
+      </c>
+      <c r="O2" s="26" t="s">
+        <v>146</v>
+      </c>
+      <c r="P2" s="26" t="s">
+        <v>148</v>
+      </c>
+      <c r="Q2" s="26" t="s">
+        <v>147</v>
+      </c>
+      <c r="R2" s="26" t="s">
+        <v>145</v>
+      </c>
+      <c r="S2" s="26" t="s">
+        <v>140</v>
+      </c>
+      <c r="T2" s="26" t="s">
+        <v>172</v>
+      </c>
+      <c r="U2" s="26" t="s">
+        <v>175</v>
+      </c>
+      <c r="V2" s="26" t="s">
+        <v>203</v>
+      </c>
+      <c r="W2" s="26" t="s">
         <v>205</v>
       </c>
-      <c r="W1" s="21" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="2" spans="1:23" s="26" customFormat="1" ht="140" x14ac:dyDescent="0.25">
-      <c r="A2" s="26" t="s">
-        <v>127</v>
-      </c>
-      <c r="B2" s="26" t="s">
-        <v>128</v>
-      </c>
-      <c r="C2" s="26" t="s">
-        <v>129</v>
-      </c>
-      <c r="D2" s="26" t="s">
-        <v>130</v>
-      </c>
-      <c r="E2" s="26" t="s">
-        <v>131</v>
-      </c>
-      <c r="F2" s="26" t="s">
-        <v>141</v>
-      </c>
-      <c r="G2" s="26" t="s">
-        <v>142</v>
-      </c>
-      <c r="H2" s="26" t="s">
-        <v>132</v>
-      </c>
-      <c r="I2" s="26" t="s">
-        <v>133</v>
-      </c>
-      <c r="J2" s="26" t="s">
-        <v>134</v>
-      </c>
-      <c r="O2" s="26" t="s">
-        <v>149</v>
-      </c>
-      <c r="P2" s="26" t="s">
-        <v>151</v>
-      </c>
-      <c r="Q2" s="26" t="s">
-        <v>150</v>
-      </c>
-      <c r="R2" s="26" t="s">
-        <v>148</v>
-      </c>
-      <c r="S2" s="26" t="s">
-        <v>143</v>
-      </c>
-      <c r="T2" s="26" t="s">
-        <v>175</v>
-      </c>
-      <c r="U2" s="26" t="s">
-        <v>178</v>
-      </c>
-      <c r="V2" s="26" t="s">
-        <v>206</v>
-      </c>
-      <c r="W2" s="26" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="X2" s="26" t="s">
+        <v>291</v>
+      </c>
+      <c r="Y2" s="26" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="3" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A3" s="25" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="B3" s="25" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="C3" s="25" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="I3" s="25" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="J3" s="25" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="K3" s="25" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="L3" s="25" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="M3" s="25" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="N3" s="25" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="O3" s="25" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="P3" s="25">
         <v>286.33</v>
@@ -2082,23 +2121,20 @@
         <v>286.33</v>
       </c>
       <c r="S3" s="25" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="T3" s="25">
         <v>123.97</v>
       </c>
       <c r="U3" s="25" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="V3" s="25" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="W3" s="25" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="H4" s="29"/>
+        <v>207</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2140,28 +2176,28 @@
         <v>82</v>
       </c>
       <c r="B1" s="21" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="C1" s="19" t="s">
         <v>67</v>
       </c>
       <c r="D1" s="18" t="s">
+        <v>149</v>
+      </c>
+      <c r="E1" s="21" t="s">
+        <v>150</v>
+      </c>
+      <c r="F1" s="21" t="s">
+        <v>151</v>
+      </c>
+      <c r="G1" s="19" t="s">
+        <v>221</v>
+      </c>
+      <c r="H1" s="19" t="s">
+        <v>220</v>
+      </c>
+      <c r="I1" s="19" t="s">
         <v>152</v>
-      </c>
-      <c r="E1" s="21" t="s">
-        <v>153</v>
-      </c>
-      <c r="F1" s="21" t="s">
-        <v>154</v>
-      </c>
-      <c r="G1" s="19" t="s">
-        <v>224</v>
-      </c>
-      <c r="H1" s="19" t="s">
-        <v>223</v>
-      </c>
-      <c r="I1" s="19" t="s">
-        <v>155</v>
       </c>
       <c r="J1" s="19" t="s">
         <v>73</v>
@@ -2205,64 +2241,64 @@
     </row>
     <row r="2" spans="1:22" s="26" customFormat="1" ht="200" x14ac:dyDescent="0.25">
       <c r="A2" s="26" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="B2" s="26" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="C2" s="26" t="s">
         <v>68</v>
       </c>
       <c r="D2" s="26" t="s">
+        <v>154</v>
+      </c>
+      <c r="E2" s="26" t="s">
+        <v>156</v>
+      </c>
+      <c r="F2" s="26" t="s">
+        <v>155</v>
+      </c>
+      <c r="G2" s="26" t="s">
+        <v>222</v>
+      </c>
+      <c r="H2" s="26" t="s">
+        <v>218</v>
+      </c>
+      <c r="I2" s="26" t="s">
+        <v>224</v>
+      </c>
+      <c r="J2" s="26" t="s">
+        <v>153</v>
+      </c>
+      <c r="K2" s="26" t="s">
         <v>157</v>
       </c>
-      <c r="E2" s="26" t="s">
+      <c r="L2" s="26" t="s">
+        <v>164</v>
+      </c>
+      <c r="M2" s="26" t="s">
+        <v>165</v>
+      </c>
+      <c r="N2" s="26" t="s">
+        <v>166</v>
+      </c>
+      <c r="O2" s="26" t="s">
+        <v>163</v>
+      </c>
+      <c r="P2" s="26" t="s">
+        <v>158</v>
+      </c>
+      <c r="Q2" s="26" t="s">
         <v>159</v>
       </c>
-      <c r="F2" s="26" t="s">
-        <v>158</v>
-      </c>
-      <c r="G2" s="26" t="s">
-        <v>225</v>
-      </c>
-      <c r="H2" s="26" t="s">
-        <v>221</v>
-      </c>
-      <c r="I2" s="26" t="s">
-        <v>227</v>
-      </c>
-      <c r="J2" s="26" t="s">
-        <v>156</v>
-      </c>
-      <c r="K2" s="26" t="s">
+      <c r="R2" s="26" t="s">
         <v>160</v>
       </c>
-      <c r="L2" s="26" t="s">
-        <v>167</v>
-      </c>
-      <c r="M2" s="26" t="s">
-        <v>168</v>
-      </c>
-      <c r="N2" s="26" t="s">
-        <v>169</v>
-      </c>
-      <c r="O2" s="26" t="s">
-        <v>166</v>
-      </c>
-      <c r="P2" s="26" t="s">
+      <c r="S2" s="26" t="s">
         <v>161</v>
       </c>
-      <c r="Q2" s="26" t="s">
+      <c r="T2" s="26" t="s">
         <v>162</v>
-      </c>
-      <c r="R2" s="26" t="s">
-        <v>163</v>
-      </c>
-      <c r="S2" s="26" t="s">
-        <v>164</v>
-      </c>
-      <c r="T2" s="26" t="s">
-        <v>165</v>
       </c>
       <c r="U2" s="26" t="s">
         <v>78</v>
@@ -2273,89 +2309,89 @@
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A3" s="25" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="B3" s="25" t="s">
+        <v>228</v>
+      </c>
+      <c r="D3" s="25" t="s">
+        <v>230</v>
+      </c>
+      <c r="E3" s="25" t="s">
         <v>231</v>
       </c>
-      <c r="D3" s="25" t="s">
-        <v>233</v>
-      </c>
-      <c r="E3" s="25" t="s">
-        <v>234</v>
-      </c>
       <c r="G3" s="25" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="H3" s="25" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="I3" s="25" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="K3" s="25">
         <v>749906</v>
       </c>
       <c r="O3" s="25" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="V3" s="25" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A4" s="25" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="I4" s="25" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="J4" s="25" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="K4" s="25">
         <v>59201</v>
       </c>
       <c r="O4" s="25" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="V4" s="25" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A5" s="25" t="s">
+        <v>233</v>
+      </c>
+      <c r="C5" s="25" t="s">
         <v>236</v>
       </c>
-      <c r="C5" s="25" t="s">
-        <v>239</v>
-      </c>
       <c r="I5" s="25" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="J5" s="25" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="K5" s="25">
         <v>74426</v>
       </c>
       <c r="O5" s="25" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="P5" s="25" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="Q5" s="25" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="R5" s="25" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="S5" s="25">
         <v>74426</v>
       </c>
       <c r="V5" s="25" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
     </row>
   </sheetData>
@@ -2391,22 +2427,22 @@
   <sheetData>
     <row r="1" spans="1:16" s="17" customFormat="1" ht="66" x14ac:dyDescent="0.25">
       <c r="A1" s="18" t="s">
+        <v>167</v>
+      </c>
+      <c r="B1" s="19" t="s">
+        <v>168</v>
+      </c>
+      <c r="C1" s="19" t="s">
         <v>170</v>
       </c>
-      <c r="B1" s="19" t="s">
-        <v>171</v>
-      </c>
-      <c r="C1" s="19" t="s">
-        <v>173</v>
-      </c>
       <c r="D1" s="18" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="E1" s="19" t="s">
         <v>88</v>
       </c>
       <c r="F1" s="19" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="G1" s="18" t="s">
         <v>89</v>
@@ -2421,7 +2457,7 @@
         <v>92</v>
       </c>
       <c r="K1" s="18" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="L1" s="18" t="s">
         <v>93</v>
@@ -2441,83 +2477,83 @@
     </row>
     <row r="2" spans="1:16" s="26" customFormat="1" ht="160" x14ac:dyDescent="0.25">
       <c r="A2" s="26" t="s">
+        <v>179</v>
+      </c>
+      <c r="B2" s="26" t="s">
+        <v>169</v>
+      </c>
+      <c r="C2" s="26" t="s">
+        <v>171</v>
+      </c>
+      <c r="F2" s="26" t="s">
+        <v>177</v>
+      </c>
+      <c r="H2" s="26" t="s">
+        <v>188</v>
+      </c>
+      <c r="I2" s="26" t="s">
+        <v>184</v>
+      </c>
+      <c r="J2" s="26" t="s">
+        <v>185</v>
+      </c>
+      <c r="K2" s="26" t="s">
+        <v>187</v>
+      </c>
+      <c r="L2" s="26" t="s">
+        <v>186</v>
+      </c>
+      <c r="M2" s="26" t="s">
+        <v>183</v>
+      </c>
+      <c r="N2" s="26" t="s">
         <v>182</v>
       </c>
-      <c r="B2" s="26" t="s">
-        <v>172</v>
-      </c>
-      <c r="C2" s="26" t="s">
-        <v>174</v>
-      </c>
-      <c r="F2" s="26" t="s">
+      <c r="O2" s="26" t="s">
+        <v>181</v>
+      </c>
+      <c r="P2" s="26" t="s">
         <v>180</v>
-      </c>
-      <c r="H2" s="26" t="s">
-        <v>191</v>
-      </c>
-      <c r="I2" s="26" t="s">
-        <v>187</v>
-      </c>
-      <c r="J2" s="26" t="s">
-        <v>188</v>
-      </c>
-      <c r="K2" s="26" t="s">
-        <v>190</v>
-      </c>
-      <c r="L2" s="26" t="s">
-        <v>189</v>
-      </c>
-      <c r="M2" s="26" t="s">
-        <v>186</v>
-      </c>
-      <c r="N2" s="26" t="s">
-        <v>185</v>
-      </c>
-      <c r="O2" s="26" t="s">
-        <v>184</v>
-      </c>
-      <c r="P2" s="26" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" s="25" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="B3" s="25" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="C3" s="25" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D3" s="25">
         <v>37</v>
       </c>
       <c r="E3" s="25" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="F3" s="25" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="J3" s="25">
         <v>24</v>
       </c>
       <c r="K3" s="25" t="s">
+        <v>246</v>
+      </c>
+      <c r="L3" s="25" t="s">
+        <v>247</v>
+      </c>
+      <c r="O3" s="25" t="s">
         <v>249</v>
       </c>
-      <c r="L3" s="25" t="s">
-        <v>250</v>
-      </c>
-      <c r="O3" s="25" t="s">
-        <v>252</v>
-      </c>
       <c r="P3" s="25" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="D12" s="31"/>
-      <c r="E12" s="31"/>
+      <c r="D12" s="30"/>
+      <c r="E12" s="30"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2526,7 +2562,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BF42104-15CD-5543-889B-11D3F56C9B51}">
-  <dimension ref="A1:R7"/>
+  <dimension ref="A1:T7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="24.6640625" style="25" customWidth="1"/>
@@ -2539,16 +2575,17 @@
     <col min="9" max="9" width="22.83203125" style="25" customWidth="1"/>
     <col min="10" max="11" width="50.33203125" style="25" customWidth="1"/>
     <col min="12" max="14" width="39.83203125" style="25" customWidth="1"/>
-    <col min="15" max="15" width="29.5" style="25" customWidth="1"/>
-    <col min="16" max="16" width="42.1640625" style="25" customWidth="1"/>
-    <col min="17" max="17" width="44.5" style="25" customWidth="1"/>
-    <col min="18" max="18" width="61" style="25" customWidth="1"/>
-    <col min="19" max="16384" width="10.83203125" style="25"/>
+    <col min="15" max="16" width="29.5" style="25" customWidth="1"/>
+    <col min="17" max="17" width="42.1640625" style="25" customWidth="1"/>
+    <col min="18" max="18" width="44.5" style="25" customWidth="1"/>
+    <col min="19" max="19" width="61" style="25" customWidth="1"/>
+    <col min="20" max="20" width="27.83203125" style="25" customWidth="1"/>
+    <col min="21" max="16384" width="10.83203125" style="25"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" s="17" customFormat="1" ht="22" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" s="17" customFormat="1" ht="22" x14ac:dyDescent="0.25">
       <c r="A1" s="21" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B1" s="18" t="s">
         <v>1</v>
@@ -2557,270 +2594,285 @@
         <v>0</v>
       </c>
       <c r="D1" s="18" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E1" s="19" t="s">
+        <v>103</v>
+      </c>
+      <c r="F1" s="19" t="s">
         <v>104</v>
       </c>
-      <c r="F1" s="19" t="s">
+      <c r="G1" s="19" t="s">
+        <v>110</v>
+      </c>
+      <c r="H1" s="21" t="s">
+        <v>106</v>
+      </c>
+      <c r="I1" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="J1" s="19" t="s">
         <v>105</v>
       </c>
-      <c r="G1" s="19" t="s">
-        <v>113</v>
-      </c>
-      <c r="H1" s="21" t="s">
-        <v>109</v>
-      </c>
-      <c r="I1" s="19" t="s">
-        <v>110</v>
-      </c>
-      <c r="J1" s="19" t="s">
-        <v>106</v>
-      </c>
       <c r="K1" s="21" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="L1" s="21" t="s">
+        <v>193</v>
+      </c>
+      <c r="M1" s="21" t="s">
+        <v>194</v>
+      </c>
+      <c r="N1" s="21" t="s">
         <v>196</v>
       </c>
-      <c r="M1" s="21" t="s">
-        <v>197</v>
-      </c>
-      <c r="N1" s="21" t="s">
-        <v>199</v>
-      </c>
       <c r="O1" s="21" t="s">
-        <v>97</v>
+        <v>286</v>
       </c>
       <c r="P1" s="21" t="s">
-        <v>99</v>
+        <v>287</v>
       </c>
       <c r="Q1" s="21" t="s">
         <v>98</v>
       </c>
-      <c r="R1" s="30" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="2" spans="1:18" s="26" customFormat="1" ht="140" x14ac:dyDescent="0.25">
+      <c r="R1" s="21" t="s">
+        <v>97</v>
+      </c>
+      <c r="S1" s="29" t="s">
+        <v>108</v>
+      </c>
+      <c r="T1" s="21" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20" s="26" customFormat="1" ht="180" x14ac:dyDescent="0.25">
       <c r="A2" s="26" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B2" s="26" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C2" s="26" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="D2" s="26" t="s">
+        <v>101</v>
+      </c>
+      <c r="E2" s="26" t="s">
+        <v>283</v>
+      </c>
+      <c r="F2" s="26" t="s">
+        <v>282</v>
+      </c>
+      <c r="G2" s="26" t="s">
+        <v>190</v>
+      </c>
+      <c r="H2" s="26" t="s">
+        <v>191</v>
+      </c>
+      <c r="I2" s="26" t="s">
+        <v>189</v>
+      </c>
+      <c r="J2" s="26" t="s">
+        <v>254</v>
+      </c>
+      <c r="K2" s="26" t="s">
+        <v>197</v>
+      </c>
+      <c r="L2" s="26" t="s">
+        <v>198</v>
+      </c>
+      <c r="M2" s="26" t="s">
+        <v>195</v>
+      </c>
+      <c r="N2" s="26" t="s">
+        <v>199</v>
+      </c>
+      <c r="O2" s="26" t="s">
+        <v>288</v>
+      </c>
+      <c r="P2" s="26" t="s">
+        <v>289</v>
+      </c>
+      <c r="Q2" s="26" t="s">
+        <v>99</v>
+      </c>
+      <c r="R2" s="26" t="s">
         <v>102</v>
       </c>
-      <c r="E2" s="26" t="s">
-        <v>107</v>
-      </c>
-      <c r="F2" s="26" t="s">
-        <v>108</v>
-      </c>
-      <c r="G2" s="26" t="s">
-        <v>193</v>
-      </c>
-      <c r="H2" s="26" t="s">
-        <v>194</v>
-      </c>
-      <c r="I2" s="26" t="s">
-        <v>192</v>
-      </c>
-      <c r="J2" s="26" t="s">
+      <c r="S2" s="26" t="s">
+        <v>109</v>
+      </c>
+      <c r="T2" s="26" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A3" s="25" t="s">
+        <v>260</v>
+      </c>
+      <c r="B3" s="25" t="s">
+        <v>258</v>
+      </c>
+      <c r="C3" s="25" t="s">
+        <v>259</v>
+      </c>
+      <c r="D3" s="25" t="s">
+        <v>229</v>
+      </c>
+      <c r="E3" s="25" t="s">
         <v>257</v>
       </c>
-      <c r="K2" s="26" t="s">
-        <v>200</v>
-      </c>
-      <c r="L2" s="26" t="s">
-        <v>201</v>
-      </c>
-      <c r="M2" s="26" t="s">
-        <v>198</v>
-      </c>
-      <c r="N2" s="26" t="s">
-        <v>202</v>
-      </c>
-      <c r="P2" s="26" t="s">
-        <v>100</v>
-      </c>
-      <c r="Q2" s="26" t="s">
-        <v>103</v>
-      </c>
-      <c r="R2" s="26" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A3" s="25" t="s">
+      <c r="J3" s="25" t="s">
+        <v>253</v>
+      </c>
+      <c r="K3" s="25" t="s">
+        <v>255</v>
+      </c>
+      <c r="Q3" s="25" t="s">
+        <v>252</v>
+      </c>
+      <c r="R3" s="25" t="s">
+        <v>251</v>
+      </c>
+      <c r="S3" s="25" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A4" s="25" t="s">
+        <v>266</v>
+      </c>
+      <c r="B4" s="25" t="s">
+        <v>265</v>
+      </c>
+      <c r="C4" s="25" t="s">
+        <v>264</v>
+      </c>
+      <c r="D4" s="25" t="s">
+        <v>262</v>
+      </c>
+      <c r="E4" s="25" t="s">
         <v>263</v>
       </c>
-      <c r="B3" s="25" t="s">
+      <c r="J4" s="25" t="s">
         <v>261</v>
       </c>
-      <c r="C3" s="25" t="s">
-        <v>262</v>
-      </c>
-      <c r="D3" s="25" t="s">
-        <v>232</v>
-      </c>
-      <c r="E3" s="25" t="s">
-        <v>260</v>
-      </c>
-      <c r="J3" s="25" t="s">
-        <v>256</v>
-      </c>
-      <c r="K3" s="25" t="s">
-        <v>258</v>
-      </c>
-      <c r="P3" s="25" t="s">
+      <c r="K4" s="25" t="s">
         <v>255</v>
       </c>
-      <c r="Q3" s="25" t="s">
-        <v>254</v>
-      </c>
-      <c r="R3" s="25" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A4" s="25" t="s">
+      <c r="R4" s="25" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A5" s="25" t="s">
+        <v>270</v>
+      </c>
+      <c r="B5" s="25" t="s">
+        <v>268</v>
+      </c>
+      <c r="C5" s="25" t="s">
         <v>269</v>
       </c>
-      <c r="B4" s="25" t="s">
-        <v>268</v>
-      </c>
-      <c r="C4" s="25" t="s">
+      <c r="D5" s="25" t="s">
+        <v>271</v>
+      </c>
+      <c r="E5" s="25" t="s">
+        <v>257</v>
+      </c>
+      <c r="J5" s="25" t="s">
         <v>267</v>
-      </c>
-      <c r="D4" s="25" t="s">
-        <v>265</v>
-      </c>
-      <c r="E4" s="25" t="s">
-        <v>266</v>
-      </c>
-      <c r="J4" s="25" t="s">
-        <v>264</v>
-      </c>
-      <c r="K4" s="25" t="s">
-        <v>258</v>
-      </c>
-      <c r="Q4" s="25" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A5" s="25" t="s">
-        <v>273</v>
-      </c>
-      <c r="B5" s="25" t="s">
-        <v>271</v>
-      </c>
-      <c r="C5" s="25" t="s">
-        <v>272</v>
-      </c>
-      <c r="D5" s="25" t="s">
-        <v>274</v>
-      </c>
-      <c r="E5" s="25" t="s">
-        <v>260</v>
-      </c>
-      <c r="J5" s="25" t="s">
-        <v>270</v>
       </c>
       <c r="K5" s="25">
         <v>619.29</v>
       </c>
-      <c r="L5" s="31" t="s">
-        <v>275</v>
+      <c r="L5" s="30" t="s">
+        <v>272</v>
       </c>
       <c r="N5" s="25">
         <v>4</v>
       </c>
-      <c r="P5" s="25" t="s">
-        <v>284</v>
-      </c>
       <c r="Q5" s="25" t="s">
-        <v>254</v>
+        <v>281</v>
       </c>
       <c r="R5" s="25" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
+        <v>251</v>
+      </c>
+      <c r="S5" s="25" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A6" s="25" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="B6" s="25" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="C6" s="25" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="D6" s="25" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="E6" s="25" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="J6" s="25" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="K6" s="25">
         <v>372.15100000000001</v>
       </c>
       <c r="L6" s="25" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="M6" s="25" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="N6" s="25">
         <v>3</v>
       </c>
-      <c r="P6" s="25" t="s">
+      <c r="Q6" s="25" t="s">
+        <v>252</v>
+      </c>
+      <c r="R6" s="25" t="s">
+        <v>251</v>
+      </c>
+      <c r="S6" s="25" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A7" s="25" t="s">
+        <v>278</v>
+      </c>
+      <c r="B7" s="25" t="s">
+        <v>279</v>
+      </c>
+      <c r="C7" s="25" t="s">
+        <v>280</v>
+      </c>
+      <c r="D7" s="25" t="s">
+        <v>271</v>
+      </c>
+      <c r="E7" s="25" t="s">
+        <v>263</v>
+      </c>
+      <c r="J7" s="25" t="s">
+        <v>277</v>
+      </c>
+      <c r="K7" s="25" t="s">
         <v>255</v>
       </c>
-      <c r="Q6" s="25" t="s">
-        <v>254</v>
-      </c>
-      <c r="R6" s="25" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A7" s="25" t="s">
-        <v>281</v>
-      </c>
-      <c r="B7" s="25" t="s">
-        <v>282</v>
-      </c>
-      <c r="C7" s="25" t="s">
-        <v>283</v>
-      </c>
-      <c r="D7" s="25" t="s">
-        <v>274</v>
-      </c>
-      <c r="E7" s="25" t="s">
-        <v>266</v>
-      </c>
-      <c r="J7" s="25" t="s">
-        <v>280</v>
-      </c>
-      <c r="K7" s="25" t="s">
-        <v>258</v>
-      </c>
-      <c r="Q7" s="25" t="s">
-        <v>254</v>
+      <c r="R7" s="25" t="s">
+        <v>251</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="R1" r:id="rId1" display="https://chembl.gitbook.io/chembl-data-deposition-guide/file-structure/field-names-and-data-types-minimal-data-submission/controlled-vocabularies/action_type-valid-names" xr:uid="{620915A2-A26D-7A4A-9BCD-73607B512014}"/>
+    <hyperlink ref="S1" r:id="rId1" display="https://chembl.gitbook.io/chembl-data-deposition-guide/file-structure/field-names-and-data-types-minimal-data-submission/controlled-vocabularies/action_type-valid-names" xr:uid="{620915A2-A26D-7A4A-9BCD-73607B512014}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>